<commit_message>
agregar etapa inicial a importar excel formato
</commit_message>
<xml_diff>
--- a/maquina.xlsx
+++ b/maquina.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Archivos Cristian\prog\Gantt-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20A50002-5F86-4045-8CE5-214239E9397D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E972976A-ECD8-49F0-85B3-E7AA6DAF7E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{27E04316-97EA-42E7-A617-05D842742A6A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="115">
   <si>
     <t>cantidad</t>
   </si>
@@ -361,6 +361,15 @@
   </si>
   <si>
     <t>PIPETA - BOMBA PITOT</t>
+  </si>
+  <si>
+    <t>etapa inicial</t>
+  </si>
+  <si>
+    <t>pedido externo</t>
+  </si>
+  <si>
+    <t>fabricacion taller</t>
   </si>
 </sst>
 </file>
@@ -443,7 +452,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -457,6 +466,7 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -772,14 +782,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13C95716-15DE-4CD7-857C-CE54B047E7DF}">
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -792,64 +803,88 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -859,8 +894,11 @@
       <c r="D9" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -868,8 +906,11 @@
         <v>12</v>
       </c>
       <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -879,8 +920,11 @@
       <c r="D11" s="3">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -890,8 +934,11 @@
       <c r="D12" s="3">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -901,8 +948,11 @@
       <c r="D13" s="3">
         <v>4.25</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -912,8 +962,11 @@
       <c r="D14" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -923,8 +976,11 @@
       <c r="D15" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
@@ -932,8 +988,11 @@
         <v>18</v>
       </c>
       <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1</v>
       </c>
@@ -943,8 +1002,11 @@
       <c r="D17" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>1</v>
       </c>
@@ -955,8 +1017,11 @@
         <f>SUM(D19:D27)</f>
         <v>12.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>1</v>
       </c>
@@ -969,8 +1034,11 @@
       <c r="D19" s="5">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>1</v>
       </c>
@@ -983,8 +1051,11 @@
       <c r="D20" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>1</v>
       </c>
@@ -995,8 +1066,11 @@
         <v>20</v>
       </c>
       <c r="D21" s="5"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>1</v>
       </c>
@@ -1007,8 +1081,11 @@
         <v>20</v>
       </c>
       <c r="D22" s="5"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>1</v>
       </c>
@@ -1021,8 +1098,11 @@
       <c r="D23" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>2</v>
       </c>
@@ -1033,8 +1113,11 @@
         <v>20</v>
       </c>
       <c r="D24" s="5"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>1</v>
       </c>
@@ -1045,8 +1128,11 @@
         <v>20</v>
       </c>
       <c r="D25" s="5"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>1</v>
       </c>
@@ -1059,8 +1145,11 @@
       <c r="D26" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>4</v>
       </c>
@@ -1071,8 +1160,11 @@
         <v>20</v>
       </c>
       <c r="D27" s="5"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1</v>
       </c>
@@ -1080,8 +1172,11 @@
         <v>30</v>
       </c>
       <c r="D28" s="3"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1</v>
       </c>
@@ -1091,8 +1186,11 @@
       <c r="D29" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1</v>
       </c>
@@ -1102,8 +1200,11 @@
       <c r="D30" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1</v>
       </c>
@@ -1113,8 +1214,11 @@
       <c r="D31" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -1122,8 +1226,11 @@
         <v>33</v>
       </c>
       <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1</v>
       </c>
@@ -1134,8 +1241,11 @@
         <f>1+8</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1</v>
       </c>
@@ -1145,8 +1255,11 @@
       <c r="D34" s="3">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1</v>
       </c>
@@ -1154,8 +1267,11 @@
         <v>36</v>
       </c>
       <c r="D35" s="3"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1</v>
       </c>
@@ -1165,8 +1281,11 @@
       <c r="D36" s="3">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1</v>
       </c>
@@ -1177,8 +1296,11 @@
         <f>3.5+0.5</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1</v>
       </c>
@@ -1188,8 +1310,11 @@
       <c r="D38" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1</v>
       </c>
@@ -1199,8 +1324,11 @@
       <c r="D39" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1</v>
       </c>
@@ -1210,8 +1338,11 @@
       <c r="D40" s="3">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E40" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>1</v>
       </c>
@@ -1222,8 +1353,11 @@
         <f>SUM(D42:D58)</f>
         <v>8.4499999999999993</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>1</v>
       </c>
@@ -1233,8 +1367,11 @@
       <c r="C42" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E42" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>1</v>
       </c>
@@ -1247,8 +1384,11 @@
       <c r="D43" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>1</v>
       </c>
@@ -1261,8 +1401,11 @@
       <c r="D44" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E44" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>1</v>
       </c>
@@ -1275,8 +1418,11 @@
       <c r="D45" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>1</v>
       </c>
@@ -1289,8 +1435,11 @@
       <c r="D46" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>1</v>
       </c>
@@ -1301,8 +1450,11 @@
         <v>42</v>
       </c>
       <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>1</v>
       </c>
@@ -1313,8 +1465,11 @@
         <v>42</v>
       </c>
       <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E48" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>2</v>
       </c>
@@ -1325,8 +1480,11 @@
         <v>42</v>
       </c>
       <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>4</v>
       </c>
@@ -1337,8 +1495,11 @@
         <v>42</v>
       </c>
       <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E50" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>2</v>
       </c>
@@ -1349,8 +1510,11 @@
         <v>42</v>
       </c>
       <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>1</v>
       </c>
@@ -1363,8 +1527,11 @@
       <c r="D52" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>2</v>
       </c>
@@ -1377,8 +1544,11 @@
       <c r="D53" s="6">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>2</v>
       </c>
@@ -1391,8 +1561,11 @@
       <c r="D54" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E54" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>1</v>
       </c>
@@ -1405,8 +1578,11 @@
       <c r="D55" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E55" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>1</v>
       </c>
@@ -1419,8 +1595,11 @@
       <c r="D56" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E56" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>2</v>
       </c>
@@ -1431,8 +1610,11 @@
         <v>42</v>
       </c>
       <c r="D57" s="6"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E57" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>6</v>
       </c>
@@ -1443,8 +1625,11 @@
         <v>42</v>
       </c>
       <c r="D58" s="6"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E58" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="7">
         <v>1</v>
       </c>
@@ -1455,8 +1640,11 @@
         <f t="shared" ref="D59" si="0">SUM(D60:D63)</f>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
         <v>1</v>
       </c>
@@ -1467,8 +1655,11 @@
         <v>59</v>
       </c>
       <c r="D60" s="9"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E60" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="7">
         <v>1</v>
       </c>
@@ -1479,8 +1670,11 @@
         <v>59</v>
       </c>
       <c r="D61" s="9"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E61" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
         <v>6</v>
       </c>
@@ -1493,8 +1687,11 @@
       <c r="D62" s="9">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E62" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="7">
         <v>6</v>
       </c>
@@ -1507,8 +1704,11 @@
       <c r="D63" s="9">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E63" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>1</v>
       </c>
@@ -1516,8 +1716,11 @@
         <v>64</v>
       </c>
       <c r="D64" s="3"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E64" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>1</v>
       </c>
@@ -1525,8 +1728,11 @@
         <v>65</v>
       </c>
       <c r="D65" s="3"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E65" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>1</v>
       </c>
@@ -1534,8 +1740,11 @@
         <v>66</v>
       </c>
       <c r="D66" s="3"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E66" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="7">
         <v>1</v>
       </c>
@@ -1545,8 +1754,11 @@
       <c r="D67" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E67" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>1</v>
       </c>
@@ -1556,8 +1768,11 @@
       <c r="D68" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E68" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>4</v>
       </c>
@@ -1567,8 +1782,11 @@
       <c r="D69" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E69" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>8</v>
       </c>
@@ -1578,8 +1796,11 @@
       <c r="D70" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E70" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>24</v>
       </c>
@@ -1587,8 +1808,11 @@
         <v>71</v>
       </c>
       <c r="D71" s="3"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>12</v>
       </c>
@@ -1598,8 +1822,11 @@
       <c r="D72" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>3</v>
       </c>
@@ -1609,8 +1836,11 @@
       <c r="D73" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E73" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>1</v>
       </c>
@@ -1620,8 +1850,11 @@
       <c r="D74" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E74" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>1</v>
       </c>
@@ -1631,8 +1864,11 @@
       <c r="D75" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E75" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>1</v>
       </c>
@@ -1642,8 +1878,11 @@
       <c r="D76" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>1</v>
       </c>
@@ -1653,8 +1892,11 @@
       <c r="D77" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E77" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>1</v>
       </c>
@@ -1664,8 +1906,11 @@
       <c r="D78" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E78" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>1</v>
       </c>
@@ -1675,8 +1920,11 @@
       <c r="D79" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E79" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>1</v>
       </c>
@@ -1687,8 +1935,11 @@
         <f t="shared" ref="D80" si="1">SUM(D81:D89)</f>
         <v>16</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E80" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>1</v>
       </c>
@@ -1701,8 +1952,11 @@
       <c r="D81" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E81" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>1</v>
       </c>
@@ -1715,8 +1969,11 @@
       <c r="D82" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E82" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>1</v>
       </c>
@@ -1729,8 +1986,11 @@
       <c r="D83" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E83" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>2</v>
       </c>
@@ -1743,8 +2003,11 @@
       <c r="D84" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E84" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>1</v>
       </c>
@@ -1757,8 +2020,11 @@
       <c r="D85" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E85" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>2</v>
       </c>
@@ -1771,8 +2037,11 @@
       <c r="D86" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E86" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
         <v>1</v>
       </c>
@@ -1785,8 +2054,11 @@
       <c r="D87" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E87" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
         <v>1</v>
       </c>
@@ -1799,8 +2071,11 @@
       <c r="D88" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E88" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
         <v>1</v>
       </c>
@@ -1813,8 +2088,11 @@
       <c r="D89" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E89" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="7">
         <v>1</v>
       </c>
@@ -1825,8 +2103,11 @@
         <f t="shared" ref="D90" si="2">SUM(D91:D100)</f>
         <v>7.4</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E90" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="7">
         <v>1</v>
       </c>
@@ -1837,8 +2118,11 @@
         <v>90</v>
       </c>
       <c r="D91" s="9"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E91" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="7">
         <v>1</v>
       </c>
@@ -1851,8 +2135,11 @@
       <c r="D92" s="9">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E92" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="7">
         <v>1</v>
       </c>
@@ -1865,8 +2152,11 @@
       <c r="D93" s="9">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="7">
         <v>1</v>
       </c>
@@ -1879,8 +2169,11 @@
       <c r="D94" s="9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="7">
         <v>1</v>
       </c>
@@ -1893,8 +2186,11 @@
       <c r="D95" s="9">
         <v>1</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E95" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="7">
         <v>1</v>
       </c>
@@ -1907,8 +2203,11 @@
       <c r="D96" s="9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E96" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="7">
         <v>1</v>
       </c>
@@ -1921,8 +2220,11 @@
       <c r="D97" s="9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="7">
         <v>1</v>
       </c>
@@ -1935,8 +2237,11 @@
       <c r="D98" s="9">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="7">
         <v>1</v>
       </c>
@@ -1949,8 +2254,11 @@
       <c r="D99" s="9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="7">
         <v>1</v>
       </c>
@@ -1963,8 +2271,11 @@
       <c r="D100" s="9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>1</v>
       </c>
@@ -1975,8 +2286,11 @@
         <f>SUM(D102:D110)</f>
         <v>4.5</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E101" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>1</v>
       </c>
@@ -1987,8 +2301,11 @@
         <v>101</v>
       </c>
       <c r="D102" s="5"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E102" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>1</v>
       </c>
@@ -2001,8 +2318,11 @@
       <c r="D103" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E103" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>2</v>
       </c>
@@ -2015,8 +2335,11 @@
       <c r="D104" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E104" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>1</v>
       </c>
@@ -2029,8 +2352,11 @@
       <c r="D105" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E105" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
         <v>1</v>
       </c>
@@ -2043,8 +2369,11 @@
       <c r="D106" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E106" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>2</v>
       </c>
@@ -2057,8 +2386,11 @@
       <c r="D107" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E107" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>1</v>
       </c>
@@ -2071,8 +2403,11 @@
       <c r="D108" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E108" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>1</v>
       </c>
@@ -2085,8 +2420,11 @@
       <c r="D109" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E109" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>1</v>
       </c>
@@ -2099,8 +2437,11 @@
       <c r="D110" s="10">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E110" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="7">
         <v>1</v>
       </c>
@@ -2110,6 +2451,9 @@
       <c r="D111" s="9">
         <f t="shared" ref="D111" si="3">SUM(D112:D122)</f>
         <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mejor visualización catálogo de maquinas y despiece con buscador y páginado, en kanban hacemos una mejor clasificación de que es un ensamble y que una pieza u operación
</commit_message>
<xml_diff>
--- a/maquina.xlsx
+++ b/maquina.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Archivos Cristian\prog\Gantt-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E972976A-ECD8-49F0-85B3-E7AA6DAF7E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31B739B-F1FE-4A47-AA3E-4293CED483AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{27E04316-97EA-42E7-A617-05D842742A6A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="109">
   <si>
     <t>cantidad</t>
   </si>
@@ -87,9 +87,6 @@
     <t xml:space="preserve">ARANDELA SOP RETEN </t>
   </si>
   <si>
-    <t>FEED SIDE</t>
-  </si>
-  <si>
     <t>ENSAMBLE FEED SIDE</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>BRIDA SUJ TREN DELANTERO</t>
   </si>
   <si>
-    <t>BANCADA DECANTER</t>
-  </si>
-  <si>
     <t>ENSAMBLE BANCADA DECANTER</t>
   </si>
   <si>
@@ -204,9 +198,6 @@
     <t>SILENT FLEX SANWICH 951216-45</t>
   </si>
   <si>
-    <t>BASE BANCADA</t>
-  </si>
-  <si>
     <t>ENSAMBLE BASE BANCADA</t>
   </si>
   <si>
@@ -267,9 +258,6 @@
     <t>SECTOR PALA CONO 6</t>
   </si>
   <si>
-    <t>CAPOTA DECANTER</t>
-  </si>
-  <si>
     <t>ENSAMBLE CAPOTA</t>
   </si>
   <si>
@@ -297,9 +285,6 @@
     <t>POSTERIOR CAPOTA CORTA</t>
   </si>
   <si>
-    <t>GUARDA MOTORES</t>
-  </si>
-  <si>
     <t>ENSAMBLE GUARDA MOTORES</t>
   </si>
   <si>
@@ -328,9 +313,6 @@
   </si>
   <si>
     <t>LATERAL IZQ GUARDA MOTOR GRANDE</t>
-  </si>
-  <si>
-    <t>CAJON SALIDA ORUJOS</t>
   </si>
   <si>
     <t>ENSAMBLE CAJON ORUJOS</t>
@@ -463,10 +445,10 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -782,7 +764,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13C95716-15DE-4CD7-857C-CE54B047E7DF}">
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.140625" bestFit="1" customWidth="1"/>
@@ -803,8 +785,8 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
-        <v>112</v>
+      <c r="E1" s="10" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -815,7 +797,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -826,7 +808,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -837,7 +819,7 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -848,7 +830,7 @@
         <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -859,7 +841,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -870,7 +852,7 @@
         <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -881,7 +863,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -895,7 +877,7 @@
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -907,7 +889,7 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -921,7 +903,7 @@
         <v>2.5</v>
       </c>
       <c r="E11" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -935,7 +917,7 @@
         <v>18</v>
       </c>
       <c r="E12" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -949,7 +931,7 @@
         <v>4.25</v>
       </c>
       <c r="E13" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -963,7 +945,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -977,7 +959,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -989,7 +971,7 @@
       </c>
       <c r="D16" s="3"/>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1003,7 +985,7 @@
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1014,11 +996,10 @@
         <v>20</v>
       </c>
       <c r="D18" s="5">
-        <f>SUM(D19:D27)</f>
-        <v>12.5</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1032,10 +1013,10 @@
         <v>20</v>
       </c>
       <c r="D19" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1048,11 +1029,9 @@
       <c r="C20" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="5">
-        <v>3</v>
-      </c>
+      <c r="D20" s="5"/>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1067,7 +1046,7 @@
       </c>
       <c r="D21" s="5"/>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1080,14 +1059,16 @@
       <c r="C22" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5">
+        <v>1</v>
+      </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>25</v>
@@ -1095,16 +1076,14 @@
       <c r="C23" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="5">
-        <v>1</v>
-      </c>
+      <c r="D23" s="5"/>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>26</v>
@@ -1114,7 +1093,7 @@
       </c>
       <c r="D24" s="5"/>
       <c r="E24" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1127,14 +1106,16 @@
       <c r="C25" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="5"/>
+      <c r="D25" s="5">
+        <v>0.5</v>
+      </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>28</v>
@@ -1142,26 +1123,21 @@
       <c r="C26" t="s">
         <v>20</v>
       </c>
-      <c r="D26" s="5">
-        <v>0.5</v>
-      </c>
+      <c r="D26" s="5"/>
       <c r="E26" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
-        <v>4</v>
-      </c>
-      <c r="B27" s="4" t="s">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
         <v>29</v>
       </c>
-      <c r="C27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" s="5"/>
+      <c r="D27" s="3"/>
       <c r="E27" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1171,9 +1147,11 @@
       <c r="B28" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="3"/>
+      <c r="D28" s="3">
+        <v>1</v>
+      </c>
       <c r="E28" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1187,7 +1165,7 @@
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1195,13 +1173,13 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D30" s="3">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1211,11 +1189,9 @@
       <c r="B31" t="s">
         <v>32</v>
       </c>
-      <c r="D31" s="3">
-        <v>1</v>
-      </c>
+      <c r="D31" s="3"/>
       <c r="E31" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1225,9 +1201,12 @@
       <c r="B32" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3">
+        <f>1+8</f>
+        <v>9</v>
+      </c>
       <c r="E32" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1238,11 +1217,10 @@
         <v>34</v>
       </c>
       <c r="D33" s="3">
-        <f>1+8</f>
-        <v>9</v>
+        <v>0.5</v>
       </c>
       <c r="E33" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1252,11 +1230,9 @@
       <c r="B34" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="3">
-        <v>0.5</v>
-      </c>
+      <c r="D34" s="3"/>
       <c r="E34" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1266,9 +1242,11 @@
       <c r="B35" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="3"/>
+      <c r="D35" s="3">
+        <v>1.5</v>
+      </c>
       <c r="E35" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1279,10 +1257,11 @@
         <v>37</v>
       </c>
       <c r="D36" s="3">
-        <v>1.5</v>
+        <f>3.5+0.5</f>
+        <v>4</v>
       </c>
       <c r="E36" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1293,11 +1272,10 @@
         <v>38</v>
       </c>
       <c r="D37" s="3">
-        <f>3.5+0.5</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1308,10 +1286,10 @@
         <v>39</v>
       </c>
       <c r="D38" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E38" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1322,24 +1300,21 @@
         <v>40</v>
       </c>
       <c r="D39" s="3">
-        <v>5</v>
+        <v>1.2</v>
       </c>
       <c r="E39" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>1</v>
-      </c>
-      <c r="B40" t="s">
+      <c r="A40" s="4">
+        <v>1</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D40" s="3">
-        <v>1.2</v>
-      </c>
       <c r="E40" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1349,12 +1324,14 @@
       <c r="B41" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="C41" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="D41" s="6">
-        <f>SUM(D42:D58)</f>
-        <v>8.4499999999999993</v>
+        <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1364,11 +1341,14 @@
       <c r="B42" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C42" t="s">
-        <v>42</v>
+      <c r="C42" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D42" s="6">
+        <v>1</v>
       </c>
       <c r="E42" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1378,14 +1358,14 @@
       <c r="B43" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C43" t="s">
-        <v>42</v>
+      <c r="C43" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D43" s="6">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1395,14 +1375,14 @@
       <c r="B44" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C44" t="s">
-        <v>42</v>
+      <c r="C44" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D44" s="6">
         <v>1</v>
       </c>
       <c r="E44" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1412,14 +1392,12 @@
       <c r="B45" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C45" t="s">
-        <v>42</v>
-      </c>
-      <c r="D45" s="6">
-        <v>1</v>
-      </c>
+      <c r="C45" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D45" s="6"/>
       <c r="E45" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1429,44 +1407,42 @@
       <c r="B46" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C46" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" s="6">
-        <v>1</v>
-      </c>
+      <c r="C46" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" s="6"/>
       <c r="E46" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C47" t="s">
-        <v>42</v>
+      <c r="C47" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C48" t="s">
-        <v>42</v>
+      <c r="C48" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1476,27 +1452,29 @@
       <c r="B49" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C49" t="s">
-        <v>42</v>
+      <c r="C49" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C50" t="s">
-        <v>42</v>
-      </c>
-      <c r="D50" s="6"/>
+      <c r="C50" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D50" s="6">
+        <v>2</v>
+      </c>
       <c r="E50" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -1506,218 +1484,206 @@
       <c r="B51" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C51" t="s">
-        <v>42</v>
-      </c>
-      <c r="D51" s="6"/>
+      <c r="C51" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D51" s="6">
+        <v>0.45</v>
+      </c>
       <c r="E51" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C52" t="s">
-        <v>42</v>
+      <c r="C52" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D52" s="6">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E52" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C53" t="s">
-        <v>42</v>
+      <c r="C53" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D53" s="6">
-        <v>0.45</v>
+        <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C54" t="s">
-        <v>42</v>
+        <v>53</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="D54" s="6">
         <v>0.5</v>
       </c>
       <c r="E54" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C55" t="s">
-        <v>42</v>
-      </c>
-      <c r="D55" s="6">
-        <v>1</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D55" s="6"/>
       <c r="E55" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C56" t="s">
-        <v>42</v>
-      </c>
-      <c r="D56" s="6">
-        <v>0.5</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D56" s="6"/>
       <c r="E56" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="4">
-        <v>2</v>
-      </c>
-      <c r="B57" s="4" t="s">
+      <c r="A57" s="7">
+        <v>1</v>
+      </c>
+      <c r="B57" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C57" t="s">
-        <v>42</v>
-      </c>
-      <c r="D57" s="6"/>
+      <c r="D57" s="8"/>
       <c r="E57" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="4">
-        <v>6</v>
-      </c>
-      <c r="B58" s="4" t="s">
+      <c r="A58" s="7">
+        <v>1</v>
+      </c>
+      <c r="B58" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C58" t="s">
-        <v>42</v>
-      </c>
-      <c r="D58" s="6"/>
+      <c r="C58" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D58" s="8"/>
       <c r="E58" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B59" s="7" t="s">
         <v>59</v>
       </c>
+      <c r="C59" s="11" t="s">
+        <v>57</v>
+      </c>
       <c r="D59" s="8">
-        <f t="shared" ref="D59" si="0">SUM(D60:D63)</f>
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E59" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B60" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C60" t="s">
-        <v>59</v>
-      </c>
-      <c r="D60" s="9"/>
+      <c r="C60" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D60" s="8">
+        <v>0.2</v>
+      </c>
       <c r="E60" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="7">
-        <v>1</v>
-      </c>
-      <c r="B61" s="7" t="s">
+      <c r="A61">
+        <v>1</v>
+      </c>
+      <c r="B61" t="s">
         <v>61</v>
       </c>
-      <c r="C61" t="s">
-        <v>59</v>
-      </c>
-      <c r="D61" s="9"/>
+      <c r="D61" s="3"/>
       <c r="E61" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="7">
-        <v>6</v>
-      </c>
-      <c r="B62" s="7" t="s">
+      <c r="A62">
+        <v>1</v>
+      </c>
+      <c r="B62" t="s">
         <v>62</v>
       </c>
-      <c r="C62" t="s">
-        <v>59</v>
-      </c>
-      <c r="D62" s="9">
-        <v>0.3</v>
-      </c>
+      <c r="D62" s="3"/>
       <c r="E62" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="7">
-        <v>6</v>
-      </c>
-      <c r="B63" s="7" t="s">
+      <c r="A63">
+        <v>1</v>
+      </c>
+      <c r="B63" t="s">
         <v>63</v>
       </c>
-      <c r="C63" t="s">
-        <v>59</v>
-      </c>
-      <c r="D63" s="9">
-        <v>0.2</v>
-      </c>
+      <c r="D63" s="3"/>
       <c r="E63" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>1</v>
-      </c>
-      <c r="B64" t="s">
+      <c r="A64" s="7">
+        <v>1</v>
+      </c>
+      <c r="B64" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D64" s="3"/>
+      <c r="D64" s="8">
+        <v>16</v>
+      </c>
       <c r="E64" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -1727,54 +1693,56 @@
       <c r="B65" t="s">
         <v>65</v>
       </c>
-      <c r="D65" s="3"/>
+      <c r="D65" s="3">
+        <v>4</v>
+      </c>
       <c r="E65" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B66" t="s">
         <v>66</v>
       </c>
-      <c r="D66" s="3"/>
+      <c r="D66" s="3">
+        <v>2</v>
+      </c>
       <c r="E66" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="7">
-        <v>1</v>
-      </c>
-      <c r="B67" s="7" t="s">
+      <c r="A67">
+        <v>8</v>
+      </c>
+      <c r="B67" t="s">
         <v>67</v>
       </c>
-      <c r="D67" s="9">
-        <v>16</v>
+      <c r="D67" s="3">
+        <v>4</v>
       </c>
       <c r="E67" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B68" t="s">
         <v>68</v>
       </c>
-      <c r="D68" s="3">
-        <v>4</v>
-      </c>
+      <c r="D68" s="3"/>
       <c r="E68" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
         <v>69</v>
@@ -1783,12 +1751,12 @@
         <v>2</v>
       </c>
       <c r="E69" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B70" t="s">
         <v>70</v>
@@ -1797,38 +1765,40 @@
         <v>4</v>
       </c>
       <c r="E70" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="B71" t="s">
         <v>71</v>
       </c>
-      <c r="D71" s="3"/>
+      <c r="D71" s="3">
+        <v>4</v>
+      </c>
       <c r="E71" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B72" t="s">
         <v>72</v>
       </c>
       <c r="D72" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E72" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B73" t="s">
         <v>73</v>
@@ -1837,7 +1807,7 @@
         <v>4</v>
       </c>
       <c r="E73" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -1851,7 +1821,7 @@
         <v>4</v>
       </c>
       <c r="E74" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -1865,7 +1835,7 @@
         <v>4</v>
       </c>
       <c r="E75" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -1879,64 +1849,75 @@
         <v>4</v>
       </c>
       <c r="E76" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77">
-        <v>1</v>
-      </c>
-      <c r="B77" t="s">
+      <c r="A77" s="4">
+        <v>1</v>
+      </c>
+      <c r="B77" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D77" s="3">
-        <v>4</v>
+      <c r="C77" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D77" s="5">
+        <v>3</v>
       </c>
       <c r="E77" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78">
-        <v>1</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="A78" s="4">
+        <v>1</v>
+      </c>
+      <c r="B78" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D78" s="3">
-        <v>4</v>
+      <c r="C78" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D78" s="5">
+        <v>3</v>
       </c>
       <c r="E78" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79">
-        <v>1</v>
-      </c>
-      <c r="B79" t="s">
+      <c r="A79" s="4">
+        <v>1</v>
+      </c>
+      <c r="B79" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D79" s="3">
-        <v>4</v>
+      <c r="C79" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D79" s="5">
+        <v>3</v>
       </c>
       <c r="E79" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>80</v>
       </c>
+      <c r="C80" s="11" t="s">
+        <v>77</v>
+      </c>
       <c r="D80" s="5">
-        <f t="shared" ref="D80" si="1">SUM(D81:D89)</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E80" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -1946,31 +1927,31 @@
       <c r="B81" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C81" t="s">
-        <v>80</v>
+      <c r="C81" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="D81" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E81" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C82" t="s">
-        <v>80</v>
+      <c r="C82" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="D82" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E82" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -1980,31 +1961,31 @@
       <c r="B83" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C83" t="s">
-        <v>80</v>
+      <c r="C83" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="D83" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E83" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C84" t="s">
-        <v>80</v>
+      <c r="C84" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="D84" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -2014,82 +1995,77 @@
       <c r="B85" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C85" t="s">
-        <v>80</v>
+      <c r="C85" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="D85" s="5">
         <v>1</v>
       </c>
       <c r="E85" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="4">
-        <v>2</v>
-      </c>
-      <c r="B86" s="4" t="s">
+      <c r="A86" s="7">
+        <v>1</v>
+      </c>
+      <c r="B86" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C86" t="s">
-        <v>80</v>
-      </c>
-      <c r="D86" s="5">
-        <v>1</v>
-      </c>
+      <c r="D86" s="8"/>
       <c r="E86" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="4">
-        <v>1</v>
-      </c>
-      <c r="B87" s="4" t="s">
+      <c r="A87" s="7">
+        <v>1</v>
+      </c>
+      <c r="B87" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C87" t="s">
-        <v>80</v>
-      </c>
-      <c r="D87" s="5">
-        <v>1</v>
+      <c r="C87" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D87" s="8">
+        <v>1.2</v>
       </c>
       <c r="E87" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="4">
-        <v>1</v>
-      </c>
-      <c r="B88" s="4" t="s">
+      <c r="A88" s="7">
+        <v>1</v>
+      </c>
+      <c r="B88" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C88" t="s">
-        <v>80</v>
-      </c>
-      <c r="D88" s="5">
-        <v>1</v>
+      <c r="C88" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D88" s="8">
+        <v>1.2</v>
       </c>
       <c r="E88" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="4">
-        <v>1</v>
-      </c>
-      <c r="B89" s="4" t="s">
+      <c r="A89" s="7">
+        <v>1</v>
+      </c>
+      <c r="B89" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C89" t="s">
-        <v>80</v>
-      </c>
-      <c r="D89" s="5">
-        <v>1</v>
+      <c r="C89" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D89" s="8">
+        <v>0.5</v>
       </c>
       <c r="E89" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -2099,12 +2075,14 @@
       <c r="B90" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D90" s="9">
-        <f t="shared" ref="D90" si="2">SUM(D91:D100)</f>
-        <v>7.4</v>
+      <c r="C90" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D90" s="8">
+        <v>1</v>
       </c>
       <c r="E90" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2114,12 +2092,14 @@
       <c r="B91" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C91" t="s">
-        <v>90</v>
-      </c>
-      <c r="D91" s="9"/>
+      <c r="C91" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D91" s="8">
+        <v>0.5</v>
+      </c>
       <c r="E91" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -2129,14 +2109,14 @@
       <c r="B92" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C92" t="s">
-        <v>90</v>
-      </c>
-      <c r="D92" s="9">
-        <v>1.2</v>
+      <c r="C92" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D92" s="8">
+        <v>0.5</v>
       </c>
       <c r="E92" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -2146,14 +2126,14 @@
       <c r="B93" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C93" t="s">
-        <v>90</v>
-      </c>
-      <c r="D93" s="9">
-        <v>1.2</v>
+      <c r="C93" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D93" s="8">
+        <v>1.5</v>
       </c>
       <c r="E93" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -2163,14 +2143,14 @@
       <c r="B94" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C94" t="s">
-        <v>90</v>
-      </c>
-      <c r="D94" s="9">
+      <c r="C94" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D94" s="8">
         <v>0.5</v>
       </c>
       <c r="E94" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2180,114 +2160,111 @@
       <c r="B95" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C95" t="s">
-        <v>90</v>
-      </c>
-      <c r="D95" s="9">
-        <v>1</v>
+      <c r="C95" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D95" s="8">
+        <v>0.5</v>
       </c>
       <c r="E95" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="7">
-        <v>1</v>
-      </c>
-      <c r="B96" s="7" t="s">
+      <c r="A96" s="4">
+        <v>1</v>
+      </c>
+      <c r="B96" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C96" t="s">
-        <v>90</v>
-      </c>
-      <c r="D96" s="9">
+      <c r="D96" s="5"/>
+      <c r="E96" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>1</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C97" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D97" s="5">
         <v>0.5</v>
       </c>
-      <c r="E96" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="7">
-        <v>1</v>
-      </c>
-      <c r="B97" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C97" t="s">
-        <v>90</v>
-      </c>
-      <c r="D97" s="9">
+      <c r="E97" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>2</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C98" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D98" s="5">
         <v>0.5</v>
       </c>
-      <c r="E97" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="7">
-        <v>1</v>
-      </c>
-      <c r="B98" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C98" t="s">
-        <v>90</v>
-      </c>
-      <c r="D98" s="9">
-        <v>1.5</v>
-      </c>
       <c r="E98" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="7">
-        <v>1</v>
-      </c>
-      <c r="B99" s="7" t="s">
+      <c r="A99" s="4">
+        <v>1</v>
+      </c>
+      <c r="B99" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C99" t="s">
-        <v>90</v>
-      </c>
-      <c r="D99" s="9">
+      <c r="C99" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D99" s="5">
         <v>0.5</v>
       </c>
       <c r="E99" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="7">
-        <v>1</v>
-      </c>
-      <c r="B100" s="7" t="s">
+      <c r="A100" s="4">
+        <v>1</v>
+      </c>
+      <c r="B100" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C100" t="s">
-        <v>90</v>
-      </c>
-      <c r="D100" s="9">
+      <c r="C100" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D100" s="5">
         <v>0.5</v>
       </c>
       <c r="E100" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>101</v>
       </c>
+      <c r="C101" s="11" t="s">
+        <v>96</v>
+      </c>
       <c r="D101" s="5">
-        <f>SUM(D102:D110)</f>
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="E101" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
@@ -2297,12 +2274,14 @@
       <c r="B102" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C102" t="s">
-        <v>101</v>
-      </c>
-      <c r="D102" s="5"/>
+      <c r="C102" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D102" s="5">
+        <v>0.5</v>
+      </c>
       <c r="E102" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -2312,148 +2291,46 @@
       <c r="B103" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C103" t="s">
-        <v>101</v>
+      <c r="C103" s="11" t="s">
+        <v>96</v>
       </c>
       <c r="D103" s="5">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E103" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B104" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C104" t="s">
-        <v>101</v>
-      </c>
-      <c r="D104" s="5">
+      <c r="C104" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D104" s="9">
         <v>0.5</v>
       </c>
       <c r="E104" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="4">
-        <v>1</v>
-      </c>
-      <c r="B105" s="4" t="s">
+      <c r="A105" s="7">
+        <v>1</v>
+      </c>
+      <c r="B105" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C105" t="s">
-        <v>101</v>
-      </c>
-      <c r="D105" s="5">
-        <v>0.5</v>
+      <c r="D105" s="8">
+        <f t="shared" ref="D105" si="0">SUM(D106:D116)</f>
+        <v>0</v>
       </c>
       <c r="E105" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="4">
-        <v>1</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C106" t="s">
-        <v>101</v>
-      </c>
-      <c r="D106" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="E106" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="4">
-        <v>2</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C107" t="s">
-        <v>101</v>
-      </c>
-      <c r="D107" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="E107" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="4">
-        <v>1</v>
-      </c>
-      <c r="B108" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C108" t="s">
-        <v>101</v>
-      </c>
-      <c r="D108" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="E108" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="4">
-        <v>1</v>
-      </c>
-      <c r="B109" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C109" t="s">
-        <v>101</v>
-      </c>
-      <c r="D109" s="5">
-        <v>1</v>
-      </c>
-      <c r="E109" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="4">
-        <v>1</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C110" t="s">
-        <v>101</v>
-      </c>
-      <c r="D110" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="E110" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="7">
-        <v>1</v>
-      </c>
-      <c r="B111" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D111" s="9">
-        <f t="shared" ref="D111" si="3">SUM(D112:D122)</f>
-        <v>0</v>
-      </c>
-      <c r="E111" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>